<commit_message>
Unify school name and academic year across phone forms and exports
</commit_message>
<xml_diff>
--- a/public/نماذج-الإشراف-المبسطة.xlsx
+++ b/public/نماذج-الإشراف-المبسطة.xlsx
@@ -123,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" readingOrder="2"/>
@@ -152,6 +152,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -758,8 +761,12 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="48" customHeight="1">
-      <c r="A3" s="10" t="n"/>
+    <row r="3" ht="76" customHeight="1">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>مدرسة عمار بن ياسر المتوسطة للبنين</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="9" t="inlineStr">
@@ -779,7 +786,11 @@
       </c>
     </row>
     <row r="7" ht="48" customHeight="1">
-      <c r="A7" s="10" t="n"/>
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>٢٠٢٦/٢٠٢٧</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add daily, staffing and late-student forms with official export headers
</commit_message>
<xml_diff>
--- a/public/نماذج-الإشراف-المبسطة.xlsx
+++ b/public/نماذج-الإشراف-المبسطة.xlsx
@@ -15,8 +15,8 @@
     <definedName name="Incidents">'القوائم'!$A$2:$A$17</definedName>
     <definedName name="Actions">'القوائم'!$B$2:$B$13</definedName>
     <definedName name="Classes">'القوائم'!$C$2:$C$41</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'الحالات'!$1:$4</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'الحالات'!$A$1:$F$16</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'الحالات'!$1:$5</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'الحالات'!$A$1:$F$17</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'الإعدادات'!$A$1:$A$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,7 +28,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -71,6 +71,23 @@
     <font>
       <name val="Arial"/>
       <sz val="16"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00303530"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00303530"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00303530"/>
+      <sz val="20"/>
     </font>
   </fonts>
   <fills count="6">
@@ -123,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" readingOrder="2"/>
@@ -152,6 +169,15 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
@@ -233,8 +259,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Cases" displayName="Cases" ref="A4:F16" headerRowCount="1">
-  <autoFilter ref="A4:F16"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Cases" displayName="Cases" ref="A5:F17" headerRowCount="1">
+  <autoFilter ref="A5:F17"/>
   <tableColumns count="6">
     <tableColumn id="1" name="التاريخ"/>
     <tableColumn id="2" name="اسم الطالب"/>
@@ -536,8 +562,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="33" customWidth="1" min="2" max="2"/>
@@ -547,66 +573,76 @@
     <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="42" customHeight="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>وزارة التربية</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>مدرسة عمار بن ياسر المتوسطة للبنين</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>منطقة الفروانية التعليمية</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
+        <is>
+          <t>العام الدراسي: ٢٠٢٦/٢٠٢٧</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="40" customHeight="1">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>سجل الحالات والمتابعة</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="32" customHeight="1">
-      <c r="A2" s="2">
-        <f>IF('الإعدادات'!A3="","اسم المدرسة",'الإعدادات'!A3)</f>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="12">
+        <f>"اسم المشرف: "&amp;IF('الإعدادات'!A5="","",'الإعدادات'!A5)</f>
         <v/>
       </c>
     </row>
-    <row r="3" ht="32" customHeight="1">
-      <c r="A3" s="2">
-        <f>"المشرف: "&amp;IF('الإعدادات'!A5="","",'الإعدادات'!A5)&amp;"    العام الدراسي: "&amp;IF('الإعدادات'!A7="","",'الإعدادات'!A7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>التاريخ</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>اسم الطالب</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>الشعبة</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>نوع الواقعة</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>الإجراء المتخذ</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>موعد المتابعة</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="4" t="n"/>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="4" t="n"/>
-    </row>
-    <row r="6" ht="36" customHeight="1">
+    <row r="6" ht="32" customHeight="1">
       <c r="A6" s="6" t="n"/>
       <c r="B6" s="7" t="n"/>
       <c r="C6" s="7" t="n"/>
@@ -614,7 +650,7 @@
       <c r="E6" s="7" t="n"/>
       <c r="F6" s="6" t="n"/>
     </row>
-    <row r="7" ht="36" customHeight="1">
+    <row r="7" ht="32" customHeight="1">
       <c r="A7" s="4" t="n"/>
       <c r="B7" s="5" t="n"/>
       <c r="C7" s="5" t="n"/>
@@ -622,7 +658,7 @@
       <c r="E7" s="5" t="n"/>
       <c r="F7" s="4" t="n"/>
     </row>
-    <row r="8" ht="36" customHeight="1">
+    <row r="8" ht="32" customHeight="1">
       <c r="A8" s="6" t="n"/>
       <c r="B8" s="7" t="n"/>
       <c r="C8" s="7" t="n"/>
@@ -630,7 +666,7 @@
       <c r="E8" s="7" t="n"/>
       <c r="F8" s="6" t="n"/>
     </row>
-    <row r="9" ht="36" customHeight="1">
+    <row r="9" ht="32" customHeight="1">
       <c r="A9" s="4" t="n"/>
       <c r="B9" s="5" t="n"/>
       <c r="C9" s="5" t="n"/>
@@ -638,7 +674,7 @@
       <c r="E9" s="5" t="n"/>
       <c r="F9" s="4" t="n"/>
     </row>
-    <row r="10" ht="36" customHeight="1">
+    <row r="10" ht="32" customHeight="1">
       <c r="A10" s="6" t="n"/>
       <c r="B10" s="7" t="n"/>
       <c r="C10" s="7" t="n"/>
@@ -646,7 +682,7 @@
       <c r="E10" s="7" t="n"/>
       <c r="F10" s="6" t="n"/>
     </row>
-    <row r="11" ht="36" customHeight="1">
+    <row r="11" ht="32" customHeight="1">
       <c r="A11" s="4" t="n"/>
       <c r="B11" s="5" t="n"/>
       <c r="C11" s="5" t="n"/>
@@ -654,7 +690,7 @@
       <c r="E11" s="5" t="n"/>
       <c r="F11" s="4" t="n"/>
     </row>
-    <row r="12" ht="36" customHeight="1">
+    <row r="12" ht="32" customHeight="1">
       <c r="A12" s="6" t="n"/>
       <c r="B12" s="7" t="n"/>
       <c r="C12" s="7" t="n"/>
@@ -662,7 +698,7 @@
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="6" t="n"/>
     </row>
-    <row r="13" ht="36" customHeight="1">
+    <row r="13" ht="32" customHeight="1">
       <c r="A13" s="4" t="n"/>
       <c r="B13" s="5" t="n"/>
       <c r="C13" s="5" t="n"/>
@@ -670,7 +706,7 @@
       <c r="E13" s="5" t="n"/>
       <c r="F13" s="4" t="n"/>
     </row>
-    <row r="14" ht="36" customHeight="1">
+    <row r="14" ht="32" customHeight="1">
       <c r="A14" s="6" t="n"/>
       <c r="B14" s="7" t="n"/>
       <c r="C14" s="7" t="n"/>
@@ -678,7 +714,7 @@
       <c r="E14" s="7" t="n"/>
       <c r="F14" s="6" t="n"/>
     </row>
-    <row r="15" ht="36" customHeight="1">
+    <row r="15" ht="32" customHeight="1">
       <c r="A15" s="4" t="n"/>
       <c r="B15" s="5" t="n"/>
       <c r="C15" s="5" t="n"/>
@@ -686,7 +722,7 @@
       <c r="E15" s="5" t="n"/>
       <c r="F15" s="4" t="n"/>
     </row>
-    <row r="16" ht="36" customHeight="1">
+    <row r="16" ht="32" customHeight="1">
       <c r="A16" s="6" t="n"/>
       <c r="B16" s="7" t="n"/>
       <c r="C16" s="7" t="n"/>
@@ -694,28 +730,39 @@
       <c r="E16" s="7" t="n"/>
       <c r="F16" s="6" t="n"/>
     </row>
+    <row r="17" ht="32" customHeight="1">
+      <c r="A17" s="4" t="n"/>
+      <c r="B17" s="5" t="n"/>
+      <c r="C17" s="5" t="n"/>
+      <c r="D17" s="5" t="n"/>
+      <c r="E17" s="5" t="n"/>
+      <c r="F17" s="4" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="6">
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A1:C1"/>
     <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="A2:C2"/>
   </mergeCells>
   <dataValidations count="5">
-    <dataValidation sqref="A5:A1004" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="date" operator="between">
+    <dataValidation sqref="A6:A1005" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date" operator="between">
       <formula1>DATE(2020,1,1)</formula1>
       <formula2>DATE(2100,12,31)</formula2>
     </dataValidation>
-    <dataValidation sqref="F5:F1004" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="date" operator="between">
+    <dataValidation sqref="F6:F1005" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date" operator="between">
       <formula1>DATE(2020,1,1)</formula1>
       <formula2>DATE(2100,12,31)</formula2>
     </dataValidation>
-    <dataValidation sqref="C5:C1004" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="قيمة غير صالحة" error="اختر من القائمة." type="list">
+    <dataValidation sqref="C6:C1005" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Classes</formula1>
     </dataValidation>
-    <dataValidation sqref="D5:D1004" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="قيمة غير صالحة" error="اختر من القائمة." type="list">
+    <dataValidation sqref="D6:D1005" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>=Incidents</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E1004" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="قيمة غير صالحة" error="اختر من القائمة." type="list">
+    <dataValidation sqref="E6:E1005" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>=Actions</formula1>
     </dataValidation>
   </dataValidations>
@@ -742,7 +789,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:A7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
   </cols>
@@ -762,7 +809,7 @@
       </c>
     </row>
     <row r="3" ht="76" customHeight="1">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>مدرسة عمار بن ياسر المتوسطة للبنين</t>
         </is>

</xml_diff>